<commit_message>
chore: sync WIP — guide-cover route, listing filters, inventories
WIP checkpoint pushed at user request. Includes: guide-cover OG/cover route
(apps/web/src/app/guide-cover/[slug] + lib/guide-cover), events/newsroom/
webinars filter + grid tweaks, GuideCard, HeaderScrollShell, importMap +
payload-types regen, package.json/pnpm-lock, dump-guides script, and the
guides/media/newsroom inventory spreadsheets. Removes AgentationDev + the
stale website-review xlsx.
</commit_message>
<xml_diff>
--- a/newsroom-data.xlsx
+++ b/newsroom-data.xlsx
@@ -467,7 +467,7 @@
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="78" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
@@ -510,7 +510,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>https://www.cleanstart.com/news/recognition-meets-real-world-detection</t>
+          <t>https://staging.cleanstart.com/news/recognition-meets-real-world-detection</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -531,7 +531,7 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>https://apnews.com/press-release/pr-newswire/cleanstart-launches-busybox-free-container-foundation-for-secure-deterministic-production-24d3771e73d0ada32e213cb07d28baf5</t>
+          <t>https://staging.cleanstart.com/news/cleanstart-launches-busybox-free-container-foundation-for-secure-deterministic-production</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -552,7 +552,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>https://www.cyberdefensemagazine.com/annual-editions/RSAC-2026/mobile/index.html#p=153</t>
+          <t>https://staging.cleanstart.com/news/ai-driven-code-and-the-expanding-challenge-of-release-trust</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -573,7 +573,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>https://www.cleanstart.com/news/cleanstart-launches-cleansight-to-give-enterprises-complete-visibility-into-container-risk</t>
+          <t>https://staging.cleanstart.com/news/cleanstart-launches-cleansight-to-give-enterprises-complete-visibility-into-container-risk</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -594,7 +594,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>https://www.cleanstart.com/news/cleanstart-wins-three-gold-awards-at-the-2026-cybersecurity-excellence-awards</t>
+          <t>https://staging.cleanstart.com/news/cleanstart-wins-three-gold-awards-at-the-2026-cybersecurity-excellence-awards</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/cleanstart-announces-strategic-partnership-with-sysdig-to-deliver-continuous-software-supply-chain-verification-from-build-to-runtime-302697035.html?tc=eml_cleartime</t>
+          <t>https://staging.cleanstart.com/news/cleanstart-announces-strategic-partnership-with-sysdig-to-deliver-continuous-software-supply-chain-verification-from</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -636,7 +636,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>https://techbullion.com/why-container-images-have-become-a-trust-boundary/</t>
+          <t>https://staging.cleanstart.com/news/why-container-images-have-become-a-trust-boundary</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -657,7 +657,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>https://www.channele2e.com/perspective/where-ai-fits-in-cybersecurity</t>
+          <t>https://staging.cleanstart.com/news/where-ai-fits-in-cybersecurity</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -678,7 +678,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>https://www.darkreading.com/application-security/sboms-in-2026-some-love-some-hate-much-ambivalence</t>
+          <t>https://staging.cleanstart.com/news/sboms-in-2026-some-love-some-hate-much-ambivalence</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -699,7 +699,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>https://www.cyberdefensemagazine.com/why-containers-drive-supply-chain-breaches/</t>
+          <t>https://staging.cleanstart.com/news/why-containers-drive-supply-chain-breaches-2</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>https://yourstory.com/2025/11/inside-cleanstarts-mission-to-make-software-safer-from-the-ground-up</t>
+          <t>https://staging.cleanstart.com/news/inside-cleanstarts-mission-to-make-software-safer-from-the-ground-up</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -741,7 +741,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>https://www.expresscomputer.in/news/zero-common-vulnerabilities-and-exposures-is-secure-by-default-the-future-of-cybersecurity/129576/</t>
+          <t>https://staging.cleanstart.com/news/zero-common-vulnerabilities-and-exposures-is-secure-by-default-the-future-of-cybersecurity</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -762,7 +762,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>https://www.darkreading.com/application-security/hardened-containers-eliminate-common-source-vulnerabilities</t>
+          <t>https://staging.cleanstart.com/news/hardened-containers-look-to-eliminate-common-source-of-vulnerabilities</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -783,7 +783,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>https://mediaindonesia.com/ekonomi/830567/kolaborasi-baru-untuk-perkuat-keamanan-perangkat-lunak-di-indonesia-dan-asean</t>
+          <t>https://staging.cleanstart.com/news/kolaborasi-baru-untuk-perkuat-keamanan-perangkat-lunak-di-indonesia-dan-asean</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -804,7 +804,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>https://www.cyberdefensemagazine.com/newsletters/november-2025/mobile/index.html#p=303</t>
+          <t>https://staging.cleanstart.com/news/why-containers-drive-supply-chain-breaches</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -825,7 +825,7 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/cleanstart-launches-industrys-most-comprehensive-sbom-analyzer-to-strengthen-container-security-302604731.html</t>
+          <t>https://staging.cleanstart.com/news/cleanstart-launches-industrys-most-comprehensive-sbom-analyzer-to-strengthen-container-security</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>https://nexusconnect.io/articles/enisa-warns-of-escalating-ot-threats</t>
+          <t>https://staging.cleanstart.com/news/enisa-warns-of-escalating-ot-threats</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>https://aijourn.com/ai-that-fixes-flaws-before-they-ship/</t>
+          <t>https://staging.cleanstart.com/news/ai-that-fixes-flaws-before-they-ship</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>https://cisoforum.in/beyond-zero-trust-redefining-software-security-in-the-age-of-compromised-code/</t>
+          <t>https://staging.cleanstart.com/news/beyond-zero-trust-redefining-software-security-in-the-age-of-compromised-code</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -909,7 +909,7 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>https://talkdev.com/quick-bytes/cleanstart-expands-vulnerability-free-container-image-library</t>
+          <t>https://staging.cleanstart.com/news/cleanstart-expands-vulnerability-free-container-image-library</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -930,7 +930,7 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>https://www.devopsdigest.com/cleanstart-expands-docker-hub-community-with-free-daily-updated-images</t>
+          <t>https://staging.cleanstart.com/news/cleanstart-expands-docker-hub-community-with-free-daily-updated-images</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>https://www.theleftshift.com/cleanstart-expands-docker-hub-community-with-free-daily-updated-hardened-images-for-secure-development-automated-refresh-cycle-delivers-hardened-near-zero-cve-images-developers-can-trus/</t>
+          <t>https://staging.cleanstart.com/news/cleanstart-expands-docker-hub-offerings-with-daily-updated-secure-images-for-developers</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -972,7 +972,7 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/cleanstart-expands-docker-hub-community-with-free-daily-updated-images-to-support-secure-development-302577984.html</t>
+          <t>https://staging.cleanstart.com/news/cleanstart-expands-docker-hub-community-with-free-daily-updated-images-to-support-secure-development</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -993,7 +993,7 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>https://techachievemedia.com/business-news/why-software-supply-chain-security-is-the-next-big-cyber-threat/</t>
+          <t>https://staging.cleanstart.com/news/why-software-supply-chain-security-is-the-next-big-cyber-threat</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1014,7 +1014,7 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>https://www.dqchannels.com/news/ecaps-to-distribute-cleanstart-products-to-strengthen-software-supply-chain-security-10499662</t>
+          <t>https://staging.cleanstart.com/news/ecaps-to-distribute-cleanstart-products-to-strengthen-software-supply-chain-security</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>https://smestreet.in/infocus/triam-security-rebrands-as-cleanstart-to-focus-on-software-supply-chain-9725369</t>
+          <t>https://staging.cleanstart.com/news/triam-security-rebrands-as-cleanstart-to-focus-on-software-supply-chain</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>https://www.apnnews.com/triam-security-rebrands-as-cleanstart-to-reflect-product-led-focus-on-securing-the-software-supply-chain/</t>
+          <t>https://staging.cleanstart.com/news/triam-security-rebrands-as-cleanstart-to-reflect-product-led-focus-on-securing-the-software-supply-chain-3</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1077,7 +1077,7 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>https://cisoforum.in/triam-security-rebrands-as-cleanstart-to-reflect-product-led-focus-on-securing-the-software-supply-chain/</t>
+          <t>https://staging.cleanstart.com/news/triam-security-rebrands-as-cleanstart-to-reflect-product-led-focus-on-securing-the-software-supply-chain-2</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1098,7 +1098,7 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>https://cxotoday.com/press-release/triam-security-rebrands-as-cleanstart-to-reflect-product-led-focus-on-securing-the-software-supply-chain/</t>
+          <t>https://staging.cleanstart.com/news/triam-security-rebrands-as-cleanstart-to-reflect-product-led-focus-on-securing-the-software-supply-chain</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>https://au.finance.yahoo.com/news/cleanstart-achieves-350-hardened-vulnerability-124500207.html</t>
+          <t>https://staging.cleanstart.com/news/cleanstart-achieves-350-hardened-vulnerability-free-container-images-accelerating-u-s-expansion</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1140,7 +1140,7 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>https://www.prnewswire.com/news-releases/openssf-welcomes-new-members-and-presents-golden-egg-award-302487512.html</t>
+          <t>https://staging.cleanstart.com/news/openssf-welcomes-new-members-and-presents-golden-egg-award-kqrhu</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1161,7 +1161,7 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>https://www.einpresswire.com/article/824869397/triam-security-s-cleanstart-wins-2025-cybersecurity-excellence-award</t>
+          <t>https://staging.cleanstart.com/news/cleanstart-wins-2025-cybersecurity-excellence-award</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1182,7 +1182,7 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>https://cbs4indy.com/business/press-releases/ein-presswire/824869397/triam-securitys-cleanstart-wins-2025-cybersecurity-excellence-award/</t>
+          <t>https://staging.cleanstart.com/news/triam-securitys-cleanstart-wins-2025-cybersecurity-excellence-award</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">

</xml_diff>